<commit_message>
Sync Friday B1 superset movements from latest xlsx
Ham curl slots across all 12 Friday sessions replaced with glute/posterior
chain movements (reverse hyper, glute bridge, back extension, cable kickback).

https://claude.ai/code/session_01VcErduov6kbPnxTCQtaP8s
</commit_message>
<xml_diff>
--- a/12 Week Upper Lower Program v4.xlsx
+++ b/12 Week Upper Lower Program v4.xlsx
@@ -2644,7 +2644,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Seated Hamstring Curl</t>
+          <t>Glute Bridge March (single-leg)</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -2669,7 +2669,7 @@
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>Knee-flex. Dorsiflex foot.</t>
+          <t>Unilateral glute + core. Decompressed. No ham curl overlap.</t>
         </is>
       </c>
     </row>
@@ -4525,7 +4525,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Nordic Hamstring Curl</t>
+          <t>Back Extension (45° hyper, BW or plate)</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -4540,7 +4540,7 @@
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>slow 3s</t>
+          <t>2011</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
@@ -4550,7 +4550,7 @@
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>BW eccentric. Heavy posterior. Standalone set — not in superset.</t>
+          <t>Glute + erector. Pause at top. No ham curl overlap.</t>
         </is>
       </c>
     </row>
@@ -6769,7 +6769,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>KB Swing</t>
+          <t>Cable Glute Kickback</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -6779,12 +6779,12 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>12–15</t>
+          <t>10–12</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>X010</t>
+          <t>2011</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
@@ -6794,7 +6794,7 @@
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>Hip ext + bracing. Glute lockout at top.</t>
+          <t>Pure glute isolation. No KB swing overlap with accessory.</t>
         </is>
       </c>
     </row>
@@ -8650,7 +8650,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Light Ham Curl</t>
+          <t>Light Back Extension (BW)</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -8660,7 +8660,7 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
@@ -8675,7 +8675,7 @@
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>PEAK WEEK.</t>
+          <t>PEAK WEEK. Erector + glute. Accessory covers ham curl.</t>
         </is>
       </c>
     </row>
@@ -10914,7 +10914,7 @@
       </c>
       <c r="B7" s="20" t="inlineStr">
         <is>
-          <t>Light Ham Curl</t>
+          <t>Light Glute Bridge</t>
         </is>
       </c>
       <c r="C7" s="20" t="inlineStr">
@@ -10939,7 +10939,7 @@
       </c>
       <c r="G7" s="20" t="inlineStr">
         <is>
-          <t>DELOAD.</t>
+          <t>DELOAD. Easy glute. Accessory covers ham curl.</t>
         </is>
       </c>
     </row>
@@ -12797,7 +12797,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Nordic Hamstring Curl</t>
+          <t>Reverse Hyper (loaded vs W1)</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -12812,7 +12812,7 @@
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>slow 4s</t>
+          <t>2011</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
@@ -12822,7 +12822,7 @@
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>Longer eccentric vs W3. BW controlled.</t>
+          <t>Add load vs W1. Decompressed posterior chain.</t>
         </is>
       </c>
     </row>
@@ -15065,7 +15065,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Lying Ham Curl (drop set)</t>
+          <t>Glute Bridge (weighted, plate on hips)</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -15090,7 +15090,7 @@
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>Drop 20% final set.</t>
+          <t>Floor-based glute. Different from A1 hip thrust angle.</t>
         </is>
       </c>
     </row>
@@ -16948,7 +16948,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Seated Ham Curl (paused)</t>
+          <t>Back Extension (paused at top, weighted)</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -16973,7 +16973,7 @@
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>Pause at peak flex.</t>
+          <t>Glute + erector. Pause peak contraction.</t>
         </is>
       </c>
     </row>
@@ -19187,7 +19187,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>RDL (DB, moderate — NOT BB)</t>
+          <t>Cable Glute Kickback (drop set)</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -19212,7 +19212,7 @@
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>Light DB only. Spinal erectors partially recovered by B1 position.</t>
+          <t>Drop 20% final set. Glute isolation peak.</t>
         </is>
       </c>
     </row>
@@ -21068,7 +21068,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Light Ham Curl</t>
+          <t>Light Back Extension (BW)</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -21078,7 +21078,7 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
@@ -21093,7 +21093,7 @@
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>PEAK WEEK.</t>
+          <t>PEAK WEEK. Accessory covers ham curl.</t>
         </is>
       </c>
     </row>
@@ -23332,7 +23332,7 @@
       </c>
       <c r="B7" s="20" t="inlineStr">
         <is>
-          <t>Light Ham Curl</t>
+          <t>Light Glute Bridge</t>
         </is>
       </c>
       <c r="C7" s="20" t="inlineStr">
@@ -23357,7 +23357,7 @@
       </c>
       <c r="G7" s="20" t="inlineStr">
         <is>
-          <t>DELOAD.</t>
+          <t>DELOAD. Accessory covers ham curl.</t>
         </is>
       </c>
     </row>
@@ -23714,7 +23714,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Lying Hamstring Curl</t>
+          <t>Reverse Hyper (or Hyper Bench)</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -23739,7 +23739,7 @@
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>Knee-flex. Slow negative.</t>
+          <t>Posterior chain decompressed. Different stimulus from accessory ham curl.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sync Tuesday B2 superset movements from latest xlsx
RDL/single-leg hinge slots across all 12 Tuesday sessions replaced with
glute/hamstring chain movements (Swiss ball curl, cable pull-through,
GHR, KB swing, glute bridge).

https://claude.ai/code/session_01VcErduov6kbPnxTCQtaP8s
</commit_message>
<xml_diff>
--- a/12 Week Upper Lower Program v4.xlsx
+++ b/12 Week Upper Lower Program v4.xlsx
@@ -3396,7 +3396,7 @@
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>Knee-flex isolation. Save Nordics for standalone sets.</t>
+          <t>Knee-flex isolation.</t>
         </is>
       </c>
     </row>
@@ -3470,7 +3470,7 @@
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>Hip-ext. Explosive glute snap.</t>
+          <t>Hip-ext. Explosive glute snap. No RDL pattern.</t>
         </is>
       </c>
     </row>
@@ -3482,28 +3482,28 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Sissy Squat (BW or light DB)</t>
+          <t>Seated Calf Raise</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr"/>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>3×10–12</t>
+          <t>3×15</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>2010</t>
+          <t>2011</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>75s</t>
+          <t>60s</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>Advanced terminal ext.</t>
+          <t>Soleus emphasis. Knees bent.</t>
         </is>
       </c>
     </row>
@@ -3515,18 +3515,18 @@
       </c>
       <c r="B10" s="16" t="inlineStr">
         <is>
-          <t>Single-Leg Ham Curl</t>
+          <t>DB Goblet Squat</t>
         </is>
       </c>
       <c r="C10" s="16" t="inlineStr"/>
       <c r="D10" s="16" t="inlineStr">
         <is>
-          <t>3×10/leg</t>
+          <t>3×12</t>
         </is>
       </c>
       <c r="E10" s="16" t="inlineStr">
         <is>
-          <t>2011</t>
+          <t>2010</t>
         </is>
       </c>
       <c r="F10" s="16" t="inlineStr">
@@ -3536,7 +3536,7 @@
       </c>
       <c r="G10" s="16" t="inlineStr">
         <is>
-          <t>Optional. Unilateral.</t>
+          <t>Optional. Upright quad focus.</t>
         </is>
       </c>
     </row>
@@ -4180,7 +4180,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Inverted Row (feet elevated)</t>
+          <t>DB Floor Press (neutral grip)</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -4195,7 +4195,7 @@
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>2011</t>
+          <t>2010</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
@@ -4205,7 +4205,7 @@
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>Horizontal pull BW. Note: B pairs pull+pull here for extra back volume on pull day.</t>
+          <t>Horizontal push. Tricep + chest. Corrects B2 from pull to push.</t>
         </is>
       </c>
     </row>
@@ -5326,7 +5326,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Stiff-Leg DL (DB)</t>
+          <t>Glute-Ham Raise (BW)</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -5351,7 +5351,7 @@
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>Hip-ext ham. More knee than RDL.</t>
+          <t>Hip-ext + knee-flex combo. Posterior chain without spinal hinge.</t>
         </is>
       </c>
     </row>
@@ -5363,18 +5363,18 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Split Squat (BW)</t>
+          <t>Copenhagen Plank</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr"/>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>3×12/leg</t>
+          <t>3×20s/side</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>2010</t>
+          <t>iso</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
@@ -5384,7 +5384,7 @@
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>Bodyweight. Unilateral focus.</t>
+          <t>Adductor isometric. Build to 30s.</t>
         </is>
       </c>
     </row>
@@ -5396,18 +5396,18 @@
       </c>
       <c r="B10" s="16" t="inlineStr">
         <is>
-          <t>KB Swing</t>
+          <t>Sissy Squat (BW)</t>
         </is>
       </c>
       <c r="C10" s="16" t="inlineStr"/>
       <c r="D10" s="16" t="inlineStr">
         <is>
-          <t>3×15</t>
+          <t>3×10</t>
         </is>
       </c>
       <c r="E10" s="16" t="inlineStr">
         <is>
-          <t>X010</t>
+          <t>2010</t>
         </is>
       </c>
       <c r="F10" s="16" t="inlineStr">
@@ -5417,7 +5417,7 @@
       </c>
       <c r="G10" s="16" t="inlineStr">
         <is>
-          <t>Optional. Hip-ext power.</t>
+          <t>Optional. Terminal knee ext.</t>
         </is>
       </c>
     </row>
@@ -7258,7 +7258,7 @@
       </c>
       <c r="B10" s="16" t="inlineStr">
         <is>
-          <t>Low-to-High Cable Fly</t>
+          <t>Pec Deck</t>
         </is>
       </c>
       <c r="C10" s="16" t="inlineStr"/>
@@ -7279,7 +7279,7 @@
       </c>
       <c r="G10" s="16" t="inlineStr">
         <is>
-          <t>PEAK WK OPTIONAL. Upper pec.</t>
+          <t>PEAK WK OPTIONAL. Different stimulus from B1 cable fly.</t>
         </is>
       </c>
     </row>
@@ -7570,7 +7570,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Single-Leg RDL (BW)</t>
+          <t>Light Swiss Ball Curl</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -7585,7 +7585,7 @@
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>2010</t>
+          <t>2011</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
@@ -7595,7 +7595,7 @@
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>Balance + hip ext. Light.</t>
+          <t>PEAK WEEK. Easy floor-based ham.</t>
         </is>
       </c>
     </row>
@@ -7607,13 +7607,13 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Leg Extension (drop set)</t>
+          <t>Single-Leg Calf Raise (BW)</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr"/>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>3×12 drop</t>
+          <t>2×12/side</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
@@ -7623,12 +7623,12 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>90s</t>
+          <t>60s</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>PEAK WK. Drop 20% last set.</t>
+          <t>PEAK WK. Easy calf.</t>
         </is>
       </c>
     </row>
@@ -7640,13 +7640,13 @@
       </c>
       <c r="B10" s="16" t="inlineStr">
         <is>
-          <t>RDL (light)</t>
+          <t>Light Leg Extension</t>
         </is>
       </c>
       <c r="C10" s="16" t="inlineStr"/>
       <c r="D10" s="16" t="inlineStr">
         <is>
-          <t>2×12</t>
+          <t>2×15</t>
         </is>
       </c>
       <c r="E10" s="16" t="inlineStr">
@@ -7661,7 +7661,7 @@
       </c>
       <c r="G10" s="16" t="inlineStr">
         <is>
-          <t>PEAK WK OPTIONAL.</t>
+          <t>PEAK WK OPTIONAL. Easy isolation.</t>
         </is>
       </c>
     </row>
@@ -9451,7 +9451,7 @@
       </c>
       <c r="B8" s="20" t="inlineStr">
         <is>
-          <t>Light RDL</t>
+          <t>Light Glute Bridge</t>
         </is>
       </c>
       <c r="C8" s="20" t="inlineStr">
@@ -9476,7 +9476,7 @@
       </c>
       <c r="G8" s="20" t="inlineStr">
         <is>
-          <t>DELOAD.</t>
+          <t>DELOAD. Easy hip-ext.</t>
         </is>
       </c>
     </row>
@@ -9488,13 +9488,13 @@
       </c>
       <c r="B9" s="20" t="inlineStr">
         <is>
-          <t>Light Leg Extension</t>
+          <t>Light Calf Raise</t>
         </is>
       </c>
       <c r="C9" s="20" t="inlineStr"/>
       <c r="D9" s="20" t="inlineStr">
         <is>
-          <t>2×12</t>
+          <t>2×15</t>
         </is>
       </c>
       <c r="E9" s="20" t="inlineStr">
@@ -9509,7 +9509,7 @@
       </c>
       <c r="G9" s="20" t="inlineStr">
         <is>
-          <t>DELOAD.</t>
+          <t>DELOAD. Easy movement.</t>
         </is>
       </c>
     </row>
@@ -9521,7 +9521,7 @@
       </c>
       <c r="B10" s="20" t="inlineStr">
         <is>
-          <t>Light Ham Curl</t>
+          <t>Light BW Squat</t>
         </is>
       </c>
       <c r="C10" s="20" t="inlineStr"/>
@@ -9532,7 +9532,7 @@
       </c>
       <c r="E10" s="20" t="inlineStr">
         <is>
-          <t>2011</t>
+          <t>2010</t>
         </is>
       </c>
       <c r="F10" s="20" t="inlineStr">
@@ -11715,7 +11715,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Good Morning (BB, light)</t>
+          <t>Cable Pull-Through (heavier vs W2)</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -11740,7 +11740,7 @@
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>Hip-ext. Hinge under load.</t>
+          <t>Add load vs B1. Hip-ext. No RDL overlap.</t>
         </is>
       </c>
     </row>
@@ -11752,28 +11752,28 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>DB Lateral Lunge</t>
+          <t>Tibialis Raise (wall or band)</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr"/>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>3×10/leg</t>
+          <t>3×15</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>2010</t>
+          <t>2011</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>75s</t>
+          <t>60s</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>Adductor + quad. Step wide.</t>
+          <t>Shin / tib anterior. Knee health + shin splint prevention.</t>
         </is>
       </c>
     </row>
@@ -11785,7 +11785,7 @@
       </c>
       <c r="B10" s="16" t="inlineStr">
         <is>
-          <t>Lying Ham Curl (add load vs W1)</t>
+          <t>Leg Extension (heavier)</t>
         </is>
       </c>
       <c r="C10" s="16" t="inlineStr"/>
@@ -11801,12 +11801,12 @@
       </c>
       <c r="F10" s="16" t="inlineStr">
         <is>
-          <t>60s</t>
+          <t>75s</t>
         </is>
       </c>
       <c r="G10" s="16" t="inlineStr">
         <is>
-          <t>Optional.</t>
+          <t>Optional. Add load vs B1.</t>
         </is>
       </c>
     </row>
@@ -13598,7 +13598,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Single-Leg RDL (BB)</t>
+          <t>Swiss Ball Hamstring Curl (feet elevated)</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -13608,7 +13608,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>10–12</t>
+          <t>12</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
@@ -13623,7 +13623,7 @@
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>Hip-ext. Add load B2.</t>
+          <t>Harder variation — elevated feet increase leverage.</t>
         </is>
       </c>
     </row>
@@ -13635,28 +13635,28 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Wall Sit (BW, 60s)</t>
+          <t>Adductor Machine (heavier)</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr"/>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>3×60s</t>
+          <t>3×10</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>iso</t>
+          <t>2011</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>60s</t>
+          <t>75s</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>Isometric quad. Burn.</t>
+          <t>Add load vs W2. Adductor strength.</t>
         </is>
       </c>
     </row>
@@ -13668,18 +13668,18 @@
       </c>
       <c r="B10" s="16" t="inlineStr">
         <is>
-          <t>Stiff-Leg DL (DB)</t>
+          <t>DB Walking Lunge</t>
         </is>
       </c>
       <c r="C10" s="16" t="inlineStr"/>
       <c r="D10" s="16" t="inlineStr">
         <is>
-          <t>3×12</t>
+          <t>3×10/leg</t>
         </is>
       </c>
       <c r="E10" s="16" t="inlineStr">
         <is>
-          <t>2011</t>
+          <t>2010</t>
         </is>
       </c>
       <c r="F10" s="16" t="inlineStr">
@@ -13689,7 +13689,7 @@
       </c>
       <c r="G10" s="16" t="inlineStr">
         <is>
-          <t>Optional. Hip-ext ham.</t>
+          <t>Optional. Unilateral quad volume.</t>
         </is>
       </c>
     </row>
@@ -13982,7 +13982,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Single-Leg RDL (DB)</t>
+          <t>Swiss Ball Hamstring Curl</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -14007,7 +14007,7 @@
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>Hip-ext ham. Balance focus.</t>
+          <t>Floor-based hip-ext + knee-flex. No RDL overlap.</t>
         </is>
       </c>
     </row>
@@ -14019,13 +14019,13 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Leg Extension</t>
+          <t>Standing Calf Raise</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr"/>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>3×12–15</t>
+          <t>3×15</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
@@ -14040,7 +14040,7 @@
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>VMO isolation. Slow negative.</t>
+          <t>Gastrocnemius. Full ROM — stretch at bottom.</t>
         </is>
       </c>
     </row>
@@ -14052,13 +14052,13 @@
       </c>
       <c r="B10" s="16" t="inlineStr">
         <is>
-          <t>Lying Hamstring Curl (extra)</t>
+          <t>Leg Extension</t>
         </is>
       </c>
       <c r="C10" s="16" t="inlineStr"/>
       <c r="D10" s="16" t="inlineStr">
         <is>
-          <t>3×12</t>
+          <t>3×12–15</t>
         </is>
       </c>
       <c r="E10" s="16" t="inlineStr">
@@ -14073,7 +14073,7 @@
       </c>
       <c r="G10" s="16" t="inlineStr">
         <is>
-          <t>Optional. Knee-flex.</t>
+          <t>Optional. Quad isolation.</t>
         </is>
       </c>
     </row>
@@ -15554,18 +15554,18 @@
       </c>
       <c r="B10" s="16" t="inlineStr">
         <is>
-          <t>Weighted Dip (chest lean)</t>
+          <t>Incline DB Fly</t>
         </is>
       </c>
       <c r="C10" s="16" t="inlineStr"/>
       <c r="D10" s="16" t="inlineStr">
         <is>
-          <t>3×8–10</t>
+          <t>3×10–12</t>
         </is>
       </c>
       <c r="E10" s="16" t="inlineStr">
         <is>
-          <t>2010</t>
+          <t>2011</t>
         </is>
       </c>
       <c r="F10" s="16" t="inlineStr">
@@ -15575,7 +15575,7 @@
       </c>
       <c r="G10" s="16" t="inlineStr">
         <is>
-          <t>Optional. Chest bias dip.</t>
+          <t>Optional. Different from A1 dip pattern.</t>
         </is>
       </c>
     </row>
@@ -15866,7 +15866,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>KB Single-Leg RDL</t>
+          <t>Band-Assisted GHR</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -15891,7 +15891,7 @@
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>Hip-ext balance work.</t>
+          <t>GHR with band decel. Hip-ext + knee-flex combo.</t>
         </is>
       </c>
     </row>
@@ -15903,28 +15903,28 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>BW Pistol Squat (parallette assist)</t>
+          <t>Single-Leg Calf Raise (weighted)</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr"/>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>3×6/leg</t>
+          <t>3×12/side</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>controlled</t>
+          <t>2011</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>75s</t>
+          <t>60s</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>Skill + strength.</t>
+          <t>Add load. Full stretch.</t>
         </is>
       </c>
     </row>
@@ -15936,28 +15936,28 @@
       </c>
       <c r="B10" s="16" t="inlineStr">
         <is>
-          <t>Seated Ham Curl</t>
+          <t>BW Pistol Squat (parallette assist)</t>
         </is>
       </c>
       <c r="C10" s="16" t="inlineStr"/>
       <c r="D10" s="16" t="inlineStr">
         <is>
-          <t>3×10–12</t>
+          <t>3×5/leg</t>
         </is>
       </c>
       <c r="E10" s="16" t="inlineStr">
         <is>
-          <t>2011</t>
+          <t>controlled</t>
         </is>
       </c>
       <c r="F10" s="16" t="inlineStr">
         <is>
-          <t>60s</t>
+          <t>75s</t>
         </is>
       </c>
       <c r="G10" s="16" t="inlineStr">
         <is>
-          <t>Optional.</t>
+          <t>Optional. Skill + strength.</t>
         </is>
       </c>
     </row>
@@ -17749,7 +17749,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Stiff-Leg DL (BB)</t>
+          <t>KB Swing (heavy)</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -17759,12 +17759,12 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>8–10</t>
+          <t>10–12</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>2011</t>
+          <t>X010</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
@@ -17774,7 +17774,7 @@
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>Add load vs W4.</t>
+          <t>Heaviest swing of program. Hip-ext dominant.</t>
         </is>
       </c>
     </row>
@@ -17786,18 +17786,18 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Leg Extension (paused)</t>
+          <t>Copenhagen Plank (weighted)</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr"/>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>3×10+2s</t>
+          <t>3×25s/side</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>2011</t>
+          <t>iso</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
@@ -17807,7 +17807,7 @@
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>Pause at top. VMO squeeze.</t>
+          <t>Add light plate. Adductor peak.</t>
         </is>
       </c>
     </row>
@@ -17819,28 +17819,28 @@
       </c>
       <c r="B10" s="16" t="inlineStr">
         <is>
-          <t>SL RDL (KB)</t>
+          <t>Leg Press (slow eccentric)</t>
         </is>
       </c>
       <c r="C10" s="16" t="inlineStr"/>
       <c r="D10" s="16" t="inlineStr">
         <is>
-          <t>3×10/leg</t>
+          <t>3×10</t>
         </is>
       </c>
       <c r="E10" s="16" t="inlineStr">
         <is>
-          <t>2011</t>
+          <t>3010</t>
         </is>
       </c>
       <c r="F10" s="16" t="inlineStr">
         <is>
-          <t>60s</t>
+          <t>75s</t>
         </is>
       </c>
       <c r="G10" s="16" t="inlineStr">
         <is>
-          <t>Optional. Balance focus.</t>
+          <t>Optional. Eccentric quad overload.</t>
         </is>
       </c>
     </row>
@@ -19988,7 +19988,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Single-Leg RDL (BW)</t>
+          <t>Light Cable Pull-Through</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -20003,7 +20003,7 @@
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>2010</t>
+          <t>2011</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
@@ -20013,7 +20013,7 @@
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>PEAK WEEK. Light.</t>
+          <t>PEAK WEEK. Easy hip-ext.</t>
         </is>
       </c>
     </row>
@@ -20025,18 +20025,18 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Light BW Squat</t>
+          <t>Light Calf Raise</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr"/>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>2×15</t>
+          <t>2×12</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>2010</t>
+          <t>2011</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
@@ -20046,7 +20046,7 @@
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>PEAK WK. Active recovery.</t>
+          <t>PEAK WK. Easy.</t>
         </is>
       </c>
     </row>
@@ -20058,13 +20058,13 @@
       </c>
       <c r="B10" s="16" t="inlineStr">
         <is>
-          <t>Light Ham Curl</t>
+          <t>Light Leg Extension</t>
         </is>
       </c>
       <c r="C10" s="16" t="inlineStr"/>
       <c r="D10" s="16" t="inlineStr">
         <is>
-          <t>2×10</t>
+          <t>2×12</t>
         </is>
       </c>
       <c r="E10" s="16" t="inlineStr">
@@ -21869,7 +21869,7 @@
       </c>
       <c r="B8" s="20" t="inlineStr">
         <is>
-          <t>Light RDL</t>
+          <t>Light Glute Bridge</t>
         </is>
       </c>
       <c r="C8" s="20" t="inlineStr">
@@ -21894,7 +21894,7 @@
       </c>
       <c r="G8" s="20" t="inlineStr">
         <is>
-          <t>DELOAD.</t>
+          <t>DELOAD. End of program.</t>
         </is>
       </c>
     </row>
@@ -21906,7 +21906,7 @@
       </c>
       <c r="B9" s="20" t="inlineStr">
         <is>
-          <t>Light Leg Extension</t>
+          <t>Light Calf Raise</t>
         </is>
       </c>
       <c r="C9" s="20" t="inlineStr"/>
@@ -21939,18 +21939,18 @@
       </c>
       <c r="B10" s="20" t="inlineStr">
         <is>
-          <t>Light RDL</t>
+          <t>Light BW Squat</t>
         </is>
       </c>
       <c r="C10" s="20" t="inlineStr"/>
       <c r="D10" s="20" t="inlineStr">
         <is>
-          <t>2×12</t>
+          <t>2×10</t>
         </is>
       </c>
       <c r="E10" s="20" t="inlineStr">
         <is>
-          <t>2011</t>
+          <t>2010</t>
         </is>
       </c>
       <c r="F10" s="20" t="inlineStr">
@@ -23857,7 +23857,7 @@
           <t>AB ROUTINE — 3 rounds, 60s rest between rounds:
   • Hanging Knee Raise — 3×12 [Hip flexion. Full dead hang. No swinging.]
   • Pallof Press — 3×10/side [Anti-rotation. Cable or band.]
-  • KB KB Swing (core focus) — 3×12 [KB — hip ext + anterior bracing. Squeeze glutes at top.]</t>
+  • KB Swing (core focus) — 3×12 [KB — hip ext + anterior bracing. Squeeze glutes at top.]</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr"/>
@@ -24515,7 +24515,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>RDL (BB)</t>
+          <t>Cable Pull-Through (rope)</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -24525,7 +24525,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>10–12</t>
+          <t>12</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
@@ -24540,7 +24540,7 @@
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>Hip-ext ham. Hinge, not squat.</t>
+          <t>Hip-ext. Spine neutral. Different stimulus from light-lift RDL.</t>
         </is>
       </c>
     </row>
@@ -24552,28 +24552,28 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Goblet Squat (paused)</t>
+          <t>Adductor Machine</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr"/>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>3×10</t>
+          <t>3×12</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>2010+2s</t>
+          <t>2011</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>75s</t>
+          <t>60s</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>Pause at bottom. Quad stretch.</t>
+          <t>Inner thigh. Important for squat stability.</t>
         </is>
       </c>
     </row>
@@ -24585,28 +24585,28 @@
       </c>
       <c r="B10" s="16" t="inlineStr">
         <is>
-          <t>Nordic Ham Curl</t>
+          <t>BW Split Squat</t>
         </is>
       </c>
       <c r="C10" s="16" t="inlineStr"/>
       <c r="D10" s="16" t="inlineStr">
         <is>
-          <t>3×6–8</t>
+          <t>3×10/leg</t>
         </is>
       </c>
       <c r="E10" s="16" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>2010</t>
         </is>
       </c>
       <c r="F10" s="16" t="inlineStr">
         <is>
-          <t>75s</t>
+          <t>60s</t>
         </is>
       </c>
       <c r="G10" s="16" t="inlineStr">
         <is>
-          <t>Optional. Eccentric emphasis.</t>
+          <t>Optional. Unilateral quad.</t>
         </is>
       </c>
     </row>

</xml_diff>